<commit_message>
docs: reconcile the RAG implementation plan with the code
- 36 of 83 tasks moved off "Not Started": 6 Completed, 30 In Progress, each
  with a dated note saying what exists, where, and what is still missing
- Owners filled where git history shows who built it (Sukumar: the Chroma /
  Ollama pipeline; Khavya: storage, provider switch)
- Decisions sheet gets a "Status in code" column (Chroma Cloud, Qwen
  embeddings, provider switch, etc.); the team's Status column is untouched
- Edge cases: 5 marked Mitigated with the evidence; E24 (chat context carries
  over between applications) recorded as found open

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LoanLensAI_RAG_Implementation_Plan.xlsx
+++ b/docs/LoanLensAI_RAG_Implementation_Plan.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$L$84</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Decisions'!$A$1:$G$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Decisions'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Storage &amp; Vector Options'!$A$1:$F$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Edge Cases'!$A$1:$H$31</definedName>
   </definedNames>
@@ -575,7 +575,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-02. Companion to LoanLensAI_Development_Task_Tracker.xlsx (separate on purpose).</t>
+          <t>2026-10-02. Companion to LoanLensAI_Development_Task_Tracker.xlsx (separate on purpose). Statuses reconciled with the code on 2026-10-29.</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,11 @@
       </c>
       <c r="J2" s="17" t="n"/>
       <c r="K2" s="12" t="inlineStr"/>
-      <c r="L2" s="12" t="n"/>
+      <c r="L2" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] No ADRs written; the Decisions sheet holds recommendations only. See the "Status in code" column there for what the code has already settled.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -2030,16 +2034,24 @@
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J6" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K6" s="12" t="inlineStr">
         <is>
           <t>Free tiers listed in Storage &amp; Vector Options sheet</t>
         </is>
       </c>
-      <c r="L6" s="12" t="n"/>
+      <c r="L6" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Chosen and running: Chroma Cloud as the vector store; embeddings via Chroma Cloud Qwen3-Embedding-0.6B on Render, Ollama locally (EMBEDDING_PROVIDER). embedTexts() is a real swap point; there is no VectorStore interface yet (chromaService.js is called directly).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -2184,12 +2196,20 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J9" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K9" s="12" t="inlineStr"/>
-      <c r="L9" s="12" t="n"/>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] The "Proposal vs Built" sheet in LoanLensAI_Development_Task_Tracker.xlsx covers the stack deviation (Node/Express + Claude / Ollama + Chroma vs FastAPI + Azure). The one-slide version is not made.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -2234,12 +2254,20 @@
       </c>
       <c r="I10" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J10" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J10" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K10" s="12" t="inlineStr"/>
-      <c r="L10" s="12" t="n"/>
+      <c r="L10" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] services/storage.js switches between MongoDB bytes and a private Cloudflare R2 bucket (STORAGE_PROVIDER). One module, not a formal interface with several adapters: no copy/exists/signedUrl, no Azure adapter.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -2284,16 +2312,24 @@
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J11" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
           <t>R2: 10 GB free, $0 egress (see options sheet)</t>
         </is>
       </c>
-      <c r="L11" s="12" t="n"/>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] R2 bucket support is built and /admin/storage-check proves a write/read/delete round trip. render.yaml defaults STORAGE_PROVIDER to "mongo"; confirm the live value, and that public access is blocked and versioning is on.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -2338,12 +2374,20 @@
       </c>
       <c r="I12" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J12" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J12" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K12" s="12" t="inlineStr"/>
-      <c r="L12" s="12" t="n"/>
+      <c r="L12" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] buildKey() builds keys from IDs only (applicationId, documentId, mime type) - no names or SSNs. No tenant prefix and no version number yet.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -2388,16 +2432,24 @@
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J13" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J13" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K13" s="12" t="inlineStr">
         <is>
           <t>Frees Atlas M0 (512 MB shared with all app data)</t>
         </is>
       </c>
-      <c r="L13" s="12" t="n"/>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] With STORAGE_PROVIDER=r2 the bytes go to R2 and MongoDB keeps storageKey, size, mime, sha256. The fileData field still exists (it is the default path), and uploads are buffered, not streamed.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -2442,12 +2494,20 @@
       </c>
       <c r="I14" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J14" s="17" t="n"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J14" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K14" s="12" t="inlineStr"/>
-      <c r="L14" s="12" t="n"/>
+      <c r="L14" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] GET /documents/:id/file streams the file through the server behind the same ownership check (borrower own, staff all; underwriter read-only), so the bucket never needs a public address. Short-lived signed URLs were not needed.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -2497,7 +2557,11 @@
       </c>
       <c r="J15" s="17" t="n"/>
       <c r="K15" s="12" t="inlineStr"/>
-      <c r="L15" s="12" t="n"/>
+      <c r="L15" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] No migration script. The demo environment is re-seeded instead, which the task allows.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -2542,12 +2606,20 @@
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J16" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J16" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K16" s="12" t="inlineStr"/>
-      <c r="L16" s="12" t="n"/>
+      <c r="L16" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] SHA-256 is computed at upload and stored on the Document. No blob dedupe and no same-file-under-two-applicants detection yet.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -2647,7 +2719,11 @@
       </c>
       <c r="J18" s="17" t="n"/>
       <c r="K18" s="12" t="inlineStr"/>
-      <c r="L18" s="12" t="n"/>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Only the mimetype allowlist exists (routes/documents.js). No magic-byte check, page cap or PDF sanitising.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -2697,7 +2773,11 @@
       </c>
       <c r="J19" s="17" t="n"/>
       <c r="K19" s="12" t="inlineStr"/>
-      <c r="L19" s="12" t="n"/>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Today a document can be hard-deleted (blob included). Supersede does keep the old version. No soft delete or legal hold.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -2896,12 +2976,20 @@
       </c>
       <c r="I23" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J23" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J23" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K23" s="12" t="inlineStr"/>
-      <c r="L23" s="12" t="n"/>
+      <c r="L23" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Built as a proxy in services/duplicateCheck.js: SSN last-4 + date of birth across applications (different name = identity reuse, same name = second open application). The plan calls for HMAC(pepper, full SSN) + DOB; the full SSN is not stored yet.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
@@ -3005,7 +3093,11 @@
           <t>Single place to audit and test</t>
         </is>
       </c>
-      <c r="L25" s="12" t="n"/>
+      <c r="L25" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Only helpers exist: chatAccess.js (chat scope), isStaff() and per-route ownership checks. No single can(principal, action, resource) module and no retrieval filter builder.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
@@ -3050,12 +3142,20 @@
       </c>
       <c r="I26" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J26" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J26" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K26" s="12" t="inlineStr"/>
-      <c r="L26" s="12" t="n"/>
+      <c r="L26" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Roles exist: borrower, officer, underwriter, admin (the underwriter is new). No tenant-admin role and no content audience tags (borrower | officer | internal).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
@@ -3100,12 +3200,20 @@
       </c>
       <c r="I27" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J27" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J27" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K27" s="12" t="inlineStr"/>
-      <c r="L27" s="12" t="n"/>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Application.reviewHistory is an append-only trail of review actions (credit score entry, checks run, refer, approve, decline, return). It does not log uploads, views, downloads, chat questions or retrieved chunk IDs.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
@@ -3246,16 +3354,24 @@
       </c>
       <c r="I30" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J30" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K30" s="12" t="inlineStr">
         <is>
           <t>Uses the Groq/Claude extraction provider already built</t>
         </is>
       </c>
-      <c r="L30" s="12" t="n"/>
+      <c r="L30" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Bank-statement PDFs are read page by page (services/pdfText.js, statementAnalysis.js) for transaction analysis. There is no general page-level transcript stored for chunking or citing loan documents.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
@@ -3350,12 +3466,20 @@
       </c>
       <c r="I32" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J32" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J32" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K32" s="12" t="inlineStr"/>
-      <c r="L32" s="12" t="n"/>
+      <c r="L32" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Policies are split at # / ## headings into chunks of up to ~1,200 characters with a small overlap for long paragraphs (services/policyChunker.js). Other document types (statements, tax returns) have no chunking strategy; PDF policies lose headings, so their citations show only the filename.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
@@ -3400,16 +3524,24 @@
       </c>
       <c r="I33" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J33" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J33" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K33" s="12" t="inlineStr">
         <is>
           <t>Check free quotas of the chosen embedding provider</t>
         </is>
       </c>
-      <c r="L33" s="12" t="n"/>
+      <c r="L33" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] services/embeddingClient.js: batching (RAG_EMBED_BATCH_SIZE), timeouts, vector validation, Ollama and Chroma Cloud providers. No retry/backoff or rate-limit handling; the model name is tagged on the collection, not on every vector.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
@@ -3454,12 +3586,20 @@
       </c>
       <c r="I34" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J34" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J34" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K34" s="12" t="inlineStr"/>
-      <c r="L34" s="12" t="n"/>
+      <c r="L34" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] services/chromaService.js: get-or-create collection, upsert, query, get, delete-by-id; chunk IDs are deterministic hashes so re-ingest is idempotent and stale chunks are removed. It refuses to mix embedding models in one collection. No tenantId filter: it is a single-tenant store.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
@@ -3504,12 +3644,20 @@
       </c>
       <c r="I35" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J35" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J35" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K35" s="12" t="inlineStr"/>
-      <c r="L35" s="12" t="n"/>
+      <c r="L35" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Each chunk carries documentId, sourceFile, sourceTitle, section, category, chunkIndex, contentHash, modifiedAt. Missing from the plan: tenantId, customerId, applicationId, docType, version, status, audience, page.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
@@ -3754,12 +3902,20 @@
       </c>
       <c r="I40" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J40" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J40" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K40" s="12" t="inlineStr"/>
-      <c r="L40" s="12" t="n"/>
+      <c r="L40" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Admin upload (routes/ragAdmin.js, admin role only): .md / .txt / text PDF, up to 10 files of 10 MB, list and delete. 8 files / 53 chunks are indexed on the live collection. No docx, no version/effective date/owner metadata, and no per-tenant partition.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
@@ -3809,7 +3965,11 @@
       </c>
       <c r="J41" s="17" t="n"/>
       <c r="K41" s="12" t="inlineStr"/>
-      <c r="L41" s="12" t="n"/>
+      <c r="L41" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] One shared Chroma collection, filtered only by category = loan-policy. No tenant, product-type or effective-date metadata.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
@@ -3854,12 +4014,20 @@
       </c>
       <c r="I42" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J42" s="17" t="n"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J42" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K42" s="12" t="inlineStr"/>
-      <c r="L42" s="12" t="n"/>
+      <c r="L42" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] ragOllama.js: embeds the question, fetches the 15 nearest chunks, drops any beyond RAG_MAX_DISTANCE (L2 distance 1.0, not a similarity score), removes duplicates, keeps 5. With nothing usable it answers "I could not find relevant information in the approved loan policies".</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
@@ -3958,12 +4126,20 @@
       </c>
       <c r="I44" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J44" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J44" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K44" s="12" t="inlineStr"/>
-      <c r="L44" s="12" t="n"/>
+      <c r="L44" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Sources carry document title, section, source file and chunk ID, and the UI shows source chips. No version, page or snippet, and the cited section cannot be opened yet (the policy page is a tracked task).</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
@@ -4008,12 +4184,20 @@
       </c>
       <c r="I45" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J45" s="17" t="n"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J45" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K45" s="12" t="inlineStr"/>
-      <c r="L45" s="12" t="n"/>
+      <c r="L45" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] CHAT_PROVIDER=anthropic or groq still puts the whole Mongo policy corpus (PolicyChunk) in the prompt; ollama uses Chroma retrieval. Note: admin uploads only reach Chroma, so they change answers only in ollama mode.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
@@ -4108,12 +4292,20 @@
       </c>
       <c r="I47" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J47" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J47" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K47" s="12" t="inlineStr"/>
-      <c r="L47" s="12" t="n"/>
+      <c r="L47" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] services/loanQuestionRouter.js classifies by rules into status / general / mixed / unsupported / clarification, with follow-up context from earlier user turns. No LLM classifier and no "calculation" or "loan-file content" categories.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
@@ -4158,16 +4350,24 @@
       </c>
       <c r="I48" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J48" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J48" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K48" s="12" t="inlineStr">
         <is>
           <t>Mostly exists</t>
         </is>
       </c>
-      <c r="L48" s="12" t="n"/>
+      <c r="L48" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Deterministic answers from MongoDB exist for status, missing documents, net pay, uploaded documents, amount and product (ragOllama.js) and as functions in verification.js. They are not exposed as a formal tool layer.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
@@ -4217,7 +4417,11 @@
       </c>
       <c r="J49" s="17" t="n"/>
       <c r="K49" s="12" t="inlineStr"/>
-      <c r="L49" s="12" t="n"/>
+      <c r="L49" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Not started: loan-file documents are not chunked or embedded.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
@@ -4262,12 +4466,20 @@
       </c>
       <c r="I50" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J50" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J50" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K50" s="12" t="inlineStr"/>
-      <c r="L50" s="12" t="n"/>
+      <c r="L50" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Facts such as amounts, net pay and dates are read from structured fields, not paraphrased, in the deterministic answers. There is no post-check that every number in a model-written answer appears in the evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
@@ -4312,12 +4524,20 @@
       </c>
       <c r="I51" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J51" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J51" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K51" s="12" t="inlineStr"/>
-      <c r="L51" s="12" t="n"/>
+      <c r="L51" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] The prompt receives the role and the borrower API view hides the credit score, audit trail and exception rationale (forViewer). Policy chunks have no audience tags, so every borrower can retrieve every policy chunk.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
@@ -4412,12 +4632,20 @@
       </c>
       <c r="I53" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J53" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J53" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K53" s="12" t="inlineStr"/>
-      <c r="L53" s="12" t="n"/>
+      <c r="L53" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Only the last four USER questions are sent as history, nothing is stored server-side, and the chat is pinned to the open application. The chat panel does not clear its messages when the open application changes, so earlier questions can carry over (edge case E24).</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
@@ -4458,12 +4686,20 @@
       </c>
       <c r="I54" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J54" s="17" t="n"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J54" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K54" s="12" t="inlineStr"/>
-      <c r="L54" s="12" t="n"/>
+      <c r="L54" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] services/rag.js picks the provider from CHAT_PROVIDER: anthropic (default), groq, ollama; MOCK_AI short-circuits all of them. Responses share the shape {answer, sources}; "usage" is not returned.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
@@ -4508,16 +4744,24 @@
       </c>
       <c r="I55" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J55" s="17" t="n"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J55" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K55" s="12" t="inlineStr">
         <is>
           <t>Free tier; rate limits vary by model</t>
         </is>
       </c>
-      <c r="L55" s="12" t="n"/>
+      <c r="L55" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] services/ragGroq.js (answerQuestionWithGroq) using the shared groqClient.js. It uses the whole Mongo corpus, not retrieval.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
@@ -4562,12 +4806,20 @@
       </c>
       <c r="I56" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J56" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J56" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K56" s="12" t="inlineStr"/>
-      <c r="L56" s="12" t="n"/>
+      <c r="L56" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] services/ragPromptBuilder.js builds the grounded prompt (answer only from evidence, cite, say when unsure). The prompt has no version id and nothing records which version produced an answer.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
@@ -4612,12 +4864,20 @@
       </c>
       <c r="I57" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J57" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J57" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K57" s="12" t="inlineStr"/>
-      <c r="L57" s="12" t="n"/>
+      <c r="L57" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] The prompt treats the question, history and evidence as untrusted data, never instructions; the model has no tools; questions are capped at RAG_MAX_QUESTION_CHARS. No injection test corpus yet.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
@@ -4662,12 +4922,20 @@
       </c>
       <c r="I58" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J58" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J58" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K58" s="12" t="inlineStr"/>
-      <c r="L58" s="12" t="n"/>
+      <c r="L58" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] parseGroundedAnswer() accepts only citations that map to retrieved chunks, retries once, then returns "I could not verify a relevant policy source". At least one valid citation is required; every claim is not checked individually.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
@@ -4712,12 +4980,20 @@
       </c>
       <c r="I59" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J59" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J59" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K59" s="12" t="inlineStr"/>
-      <c r="L59" s="12" t="n"/>
+      <c r="L59" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Provider calls have timeouts and abort when the client disconnects, and failures return a friendly message. No circuit breaker, no provider failover and no degraded structured-only answer.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
@@ -4858,12 +5134,20 @@
       </c>
       <c r="I62" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J62" s="17" t="n"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J62" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K62" s="12" t="inlineStr"/>
-      <c r="L62" s="12" t="n"/>
+      <c r="L62" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] data/seed/test-questions.md has 30 numbered questions across borrower, officer, small-business and refusal cases, each with the expected source. It is a manual acceptance list; nothing scores retrieval automatically yet.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
@@ -5058,12 +5342,20 @@
       </c>
       <c r="I66" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J66" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J66" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K66" s="12" t="inlineStr"/>
-      <c r="L66" s="12" t="n"/>
+      <c r="L66" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Tests exist for chat access scope, the untrusted-data prompt, forged citations, admin-only access and the borrower view hiding internals (backend/test/rag, backend/test/decisions). No cross-tenant leakage suite, injection corpus or PII probes.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
@@ -5304,12 +5596,20 @@
       </c>
       <c r="I71" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J71" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J71" s="17" t="inlineStr">
+        <is>
+          <t>Sukumar</t>
+        </is>
+      </c>
       <c r="K71" s="12" t="inlineStr"/>
-      <c r="L71" s="12" t="n"/>
+      <c r="L71" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] RAG logging records reasons and counts only, not the question or policy text. Other routes were not audited, and the audit log is not a separate restricted store.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="12" t="inlineStr">
@@ -5554,16 +5854,24 @@
       </c>
       <c r="I76" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J76" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J76" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K76" s="12" t="inlineStr">
         <is>
           <t>Source chips already exist</t>
         </is>
       </c>
-      <c r="L76" s="12" t="n"/>
+      <c r="L76" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] Done: answers with headings, bullets, highlighted next steps and coloured status words; sample questions; "Opened &lt;page&gt;" links; error states. Missing: a citations drawer that opens the cited policy, feedback buttons, index-status awareness.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
@@ -5712,12 +6020,20 @@
       </c>
       <c r="I79" s="12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J79" s="17" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J79" s="17" t="inlineStr">
+        <is>
+          <t>Khavya</t>
+        </is>
+      </c>
       <c r="K79" s="12" t="inlineStr"/>
-      <c r="L79" s="12" t="n"/>
+      <c r="L79" s="12" t="inlineStr">
+        <is>
+          <t>[2026-10-29] POST /chat/:applicationId returns {answer, sources} and only the web app calls it. Nothing about it is written down as a contract for other channels.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
@@ -6006,7 +6322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6016,6 +6332,7 @@
     <col width="56" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6054,6 +6371,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Status in code (2026-10-29)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
@@ -6091,6 +6413,11 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>Not implemented: single-bank app, no tenant model.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -6128,6 +6455,11 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>Partly: private Cloudflare R2 behind a switch (STORAGE_PROVIDER); MongoDB is still the default.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -6165,6 +6497,11 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>No code yet.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -6202,6 +6539,11 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>Partly: R2 keys are built from IDs only (no tenant prefix or version).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -6239,6 +6581,11 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>Partly: duplicateCheck.js uses SSN last-4 + date of birth (a proxy for the keyed hash the plan recommends).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -6276,6 +6623,11 @@
           <t>Needs input</t>
         </is>
       </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>In use: Chroma Cloud (collection loan-knowledge-qwen on Render). Not Atlas Vector Search, which the plan recommended.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -6313,6 +6665,11 @@
           <t>Needs input</t>
         </is>
       </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>In use: Chroma Cloud Qwen3-Embedding-0.6B on Render, Ollama nomic-embed-text locally.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -6350,6 +6707,11 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>Dense search only, fixed L2 cutoff 1.0, top 5 of 15. No hybrid or rerank.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -6387,6 +6749,11 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>In use: CHAT_PROVIDER = anthropic | groq | ollama | mock. Render runs Ollama Cloud.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -6424,6 +6791,11 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>Policy text only is embedded. The question text is sent to the embedding and chat vendors unredacted.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -6461,6 +6833,11 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>Not implemented for policy chunks (no audience tags); the borrower API view does hide internal fields.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -6498,6 +6875,11 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Policies are ingested inline in the admin upload request. No loan-file ingestion.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -6535,6 +6917,11 @@
           <t>Needs input</t>
         </is>
       </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>No code yet.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -6572,9 +6959,14 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Web only; WhatsApp not started.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G15"/>
+  <autoFilter ref="A1:H15"/>
   <conditionalFormatting sqref="G2:G100">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Decided"</formula>
@@ -7706,12 +8098,12 @@
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
-          <t>Seed two customers with same SSN hash -&gt; flagged</t>
+          <t>Seed two customers with same SSN hash -&gt; flagged [2026-10-29] duplicateCheck.js flags a later application that reuses an earlier SSN last-4 + date of birth (proxy for the keyed hash).</t>
         </is>
       </c>
       <c r="H2" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Mitigated</t>
         </is>
       </c>
     </row>
@@ -7748,12 +8140,12 @@
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Second application shares KYC doc, no copy</t>
+          <t>Second application shares KYC doc, no copy [2026-10-29] A second open application by the same person is flagged (same-person-open). Document reuse across applications is not built.</t>
         </is>
       </c>
       <c r="H3" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Mitigated</t>
         </is>
       </c>
     </row>
@@ -7832,12 +8224,12 @@
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Upload '../../x.png' -&gt; stored under ID key</t>
+          <t>Upload '../../x.png' -&gt; stored under ID key [2026-10-29] R2 keys come from IDs only (storage.js buildKey); the filename is stored as metadata.</t>
         </is>
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Mitigated</t>
         </is>
       </c>
     </row>
@@ -8126,12 +8518,12 @@
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>Adversarial prompts return refusal</t>
+          <t>Adversarial prompts return refusal [2026-10-29] Authorization is server-side (chat route + chatAccess); the model never decides who may see what.</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Mitigated</t>
         </is>
       </c>
     </row>
@@ -8420,12 +8812,12 @@
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>Out-of-scope questions refused</t>
+          <t>Out-of-scope questions refused [2026-10-29] Distance cutoff plus a "could not find relevant information" answer when nothing is retrieved (ragOllama.js).</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Mitigated</t>
         </is>
       </c>
     </row>
@@ -8672,7 +9064,7 @@
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>Switch application -&gt; context cleared</t>
+          <t>Switch application -&gt; context cleared [2026-10-29] Found open: the chat panel keeps its messages when the open application changes, so earlier questions can carry over.</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr">

</xml_diff>